<commit_message>
Receipt-X v1.1 - Admin tools, UI redesign, navigation and Product Master update
</commit_message>
<xml_diff>
--- a/RECEIPT-X_PRODUCT_MASTER.xlsx
+++ b/RECEIPT-X_PRODUCT_MASTER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\OneDrive\Desktop\Mabruk\PRODUCT_MASTER\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\OneDrive\Desktop\Mabruk\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8180" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8180" firstSheet="15" activeTab="22"/>
   </bookViews>
   <sheets>
     <sheet name="PWANI OIL PRODUCTS" sheetId="1" r:id="rId1"/>
@@ -17,9 +17,24 @@
     <sheet name="MVITA OIL" sheetId="3" r:id="rId3"/>
     <sheet name="YEMKEN" sheetId="4" r:id="rId4"/>
     <sheet name="KILIMANJARO BISCUITS" sheetId="5" r:id="rId5"/>
-    <sheet name="KENAFRIC" sheetId="6" r:id="rId6"/>
-    <sheet name="MZURI SWEETS" sheetId="14" r:id="rId7"/>
-    <sheet name="AZAM" sheetId="15" r:id="rId8"/>
+    <sheet name="DOLA" sheetId="16" r:id="rId6"/>
+    <sheet name="MOMBASA MAIZE MILLERS" sheetId="17" r:id="rId7"/>
+    <sheet name="Soft Care" sheetId="18" r:id="rId8"/>
+    <sheet name="KEVIAN KENYA" sheetId="19" r:id="rId9"/>
+    <sheet name="CHANDARIA" sheetId="20" r:id="rId10"/>
+    <sheet name="KINANGOP " sheetId="21" r:id="rId11"/>
+    <sheet name="DAIMA" sheetId="22" r:id="rId12"/>
+    <sheet name="BROOKSIDE" sheetId="23" r:id="rId13"/>
+    <sheet name="KENAFRIC" sheetId="6" r:id="rId14"/>
+    <sheet name="MZURI SWEETS" sheetId="14" r:id="rId15"/>
+    <sheet name="UJI PWANI" sheetId="24" r:id="rId16"/>
+    <sheet name="AZAM" sheetId="15" r:id="rId17"/>
+    <sheet name="MBEGU SABA" sheetId="25" r:id="rId18"/>
+    <sheet name="AYWAA" sheetId="26" r:id="rId19"/>
+    <sheet name="U-FRESH" sheetId="27" r:id="rId20"/>
+    <sheet name="ZEN MAHITAJI" sheetId="28" r:id="rId21"/>
+    <sheet name="SUGAR" sheetId="29" r:id="rId22"/>
+    <sheet name="BEANS" sheetId="30" r:id="rId23"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="188">
   <si>
     <t>Brand</t>
   </si>
@@ -181,6 +196,420 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Dola sima</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Dola Ngano</t>
+  </si>
+  <si>
+    <t>Dola Atta Mark 1 Ngano</t>
+  </si>
+  <si>
+    <t>Dola Gold</t>
+  </si>
+  <si>
+    <t>Jahazi Ngano</t>
+  </si>
+  <si>
+    <t>Jahazi Sima</t>
+  </si>
+  <si>
+    <t>Jahazi Atta Mark 1 ngano</t>
+  </si>
+  <si>
+    <t>Dola Bakers Flour</t>
+  </si>
+  <si>
+    <t>50kg</t>
+  </si>
+  <si>
+    <t>25kg</t>
+  </si>
+  <si>
+    <t>Ziwa Sima</t>
+  </si>
+  <si>
+    <t>Ziwa Ngano</t>
+  </si>
+  <si>
+    <t>Baba Lao Sima</t>
+  </si>
+  <si>
+    <t>Baba Lao Ngano</t>
+  </si>
+  <si>
+    <t>Dola Chenga</t>
+  </si>
+  <si>
+    <t>Taifa sima</t>
+  </si>
+  <si>
+    <t>Taifa  sima</t>
+  </si>
+  <si>
+    <t>Taifa Ngano</t>
+  </si>
+  <si>
+    <t>Taifa  Ngano</t>
+  </si>
+  <si>
+    <t>Taifa Atta Mark 1 Ngano</t>
+  </si>
+  <si>
+    <t>Taifa  Atta Mark 1 Ngano</t>
+  </si>
+  <si>
+    <t>Ndovu Atta Mark 1 ngano</t>
+  </si>
+  <si>
+    <t>Ndovu  Sima</t>
+  </si>
+  <si>
+    <t>Ndovu Sima</t>
+  </si>
+  <si>
+    <t>Ndovu Ngano</t>
+  </si>
+  <si>
+    <t>Tifa Chenga</t>
+  </si>
+  <si>
+    <t>Cosmo Sima</t>
+  </si>
+  <si>
+    <t>Cosmo Ngano</t>
+  </si>
+  <si>
+    <t>Swan Sima</t>
+  </si>
+  <si>
+    <t>1lt</t>
+  </si>
+  <si>
+    <t>2lt</t>
+  </si>
+  <si>
+    <t>3lt</t>
+  </si>
+  <si>
+    <t>5lt</t>
+  </si>
+  <si>
+    <t>10lt</t>
+  </si>
+  <si>
+    <t>20lt</t>
+  </si>
+  <si>
+    <t>Halisi Fry</t>
+  </si>
+  <si>
+    <t>Bora Cooking Fat</t>
+  </si>
+  <si>
+    <t>San Salt</t>
+  </si>
+  <si>
+    <t>200g</t>
+  </si>
+  <si>
+    <t>Patco Sweets</t>
+  </si>
+  <si>
+    <t>Jumbo Low Count Small</t>
+  </si>
+  <si>
+    <t>Jumbo Low Count Medium</t>
+  </si>
+  <si>
+    <t>Jumbo Low Count Large</t>
+  </si>
+  <si>
+    <t>Jumbo Low Count Extra large</t>
+  </si>
+  <si>
+    <t>Software Premium high Count Large</t>
+  </si>
+  <si>
+    <t>Software Premium high Count Medium</t>
+  </si>
+  <si>
+    <t>Software Premium high Count Small</t>
+  </si>
+  <si>
+    <t>Software Premium high Count Extra Large</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>Extra Large</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soft Care Gold Diapers High Count </t>
+  </si>
+  <si>
+    <t>Soft Care Space Diapers</t>
+  </si>
+  <si>
+    <t>Jumbo Large</t>
+  </si>
+  <si>
+    <t>Jumbo Small</t>
+  </si>
+  <si>
+    <t>High Count Medium</t>
+  </si>
+  <si>
+    <t>SoftCare Baby Pants/Gold High Count Pants</t>
+  </si>
+  <si>
+    <t>SoftCare Baby Pants/Gold High Midi Packs</t>
+  </si>
+  <si>
+    <t>SoftCare Wet Wipes</t>
+  </si>
+  <si>
+    <t>Soft Care Sanitary Pads</t>
+  </si>
+  <si>
+    <t>Maxi Thick</t>
+  </si>
+  <si>
+    <t>Model S</t>
+  </si>
+  <si>
+    <t>Extra LongSmart</t>
+  </si>
+  <si>
+    <t>Smart</t>
+  </si>
+  <si>
+    <t>200ml</t>
+  </si>
+  <si>
+    <t>Afia Mango Juice</t>
+  </si>
+  <si>
+    <t>Afia Mixed Fruit Juice</t>
+  </si>
+  <si>
+    <t>Velvex Ultra Dry Sanitary Pads</t>
+  </si>
+  <si>
+    <t>Velvet Toilet Tissue</t>
+  </si>
+  <si>
+    <t>Safari Tissue</t>
+  </si>
+  <si>
+    <t>Nice and Soft Tissue</t>
+  </si>
+  <si>
+    <t>Rosy Toilet Tissue</t>
+  </si>
+  <si>
+    <t>Wet Wipes</t>
+  </si>
+  <si>
+    <t>Kinangop Fresh Milk</t>
+  </si>
+  <si>
+    <t>Kinangop Long life Milk</t>
+  </si>
+  <si>
+    <t>Kinangop Gold Life(UHT)Milk</t>
+  </si>
+  <si>
+    <t>kinangop Gold Fresh Milk</t>
+  </si>
+  <si>
+    <t>Kinangop Gold Long Life Milk</t>
+  </si>
+  <si>
+    <t>Daima Fresh Milk (esl)</t>
+  </si>
+  <si>
+    <t>Daima Long Life(UHT)</t>
+  </si>
+  <si>
+    <t>Brookside Fresh Milk</t>
+  </si>
+  <si>
+    <t>Brookside Long Life(UHT Milk</t>
+  </si>
+  <si>
+    <t>Brookside Long Life(UHT)Milk</t>
+  </si>
+  <si>
+    <t>Azam Energy Drink Coffee Malt</t>
+  </si>
+  <si>
+    <t>Azam Energy Drink Apple Malt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azam Embe </t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Azam Tropical Mix</t>
+  </si>
+  <si>
+    <t>Azam Orange</t>
+  </si>
+  <si>
+    <t>Azam Guava</t>
+  </si>
+  <si>
+    <t>Azam Green Mango</t>
+  </si>
+  <si>
+    <t>Azam Cola Orange Splash</t>
+  </si>
+  <si>
+    <t>Azam Cola Apple Splash</t>
+  </si>
+  <si>
+    <t>Azam Cola Tangawizi</t>
+  </si>
+  <si>
+    <t>Azam Cola Swiss Soda</t>
+  </si>
+  <si>
+    <t>Azam Uhai Water</t>
+  </si>
+  <si>
+    <t>350ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azam Ukwaju </t>
+  </si>
+  <si>
+    <t>Azam Ukwaju</t>
+  </si>
+  <si>
+    <t>20x100pcs</t>
+  </si>
+  <si>
+    <t>Mr Berry Chocolate</t>
+  </si>
+  <si>
+    <t>12x50pcs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Big Daddy </t>
+  </si>
+  <si>
+    <t>Strawberry</t>
+  </si>
+  <si>
+    <t>Passion</t>
+  </si>
+  <si>
+    <t>Milk</t>
+  </si>
+  <si>
+    <t>King Kuba</t>
+  </si>
+  <si>
+    <t>King kuba</t>
+  </si>
+  <si>
+    <t>Tajiri Pops</t>
+  </si>
+  <si>
+    <t>No.1 Lollipop</t>
+  </si>
+  <si>
+    <t>Xplode</t>
+  </si>
+  <si>
+    <t>Tutti Frutti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Big Boss </t>
+  </si>
+  <si>
+    <t>Mint</t>
+  </si>
+  <si>
+    <t>Gomba</t>
+  </si>
+  <si>
+    <t>Mambo</t>
+  </si>
+  <si>
+    <t>Ice Cool</t>
+  </si>
+  <si>
+    <t>Funky Monkey Assorted</t>
+  </si>
+  <si>
+    <t>Kaboom</t>
+  </si>
+  <si>
+    <t>Kashata Krunch</t>
+  </si>
+  <si>
+    <t>Toffees</t>
+  </si>
+  <si>
+    <t>No.1</t>
+  </si>
+  <si>
+    <t>Kashata</t>
+  </si>
+  <si>
+    <t>Uji Pwani</t>
+  </si>
+  <si>
+    <t>Mbegu Saba</t>
+  </si>
+  <si>
+    <t>KT Tomato Paste</t>
+  </si>
+  <si>
+    <t>80g</t>
+  </si>
+  <si>
+    <t>Lazan Tomato Paste</t>
+  </si>
+  <si>
+    <t>U Fresh</t>
+  </si>
+  <si>
+    <t>U fresh</t>
+  </si>
+  <si>
+    <t>Pep Tang Tomato Sauce</t>
+  </si>
+  <si>
+    <t>20g</t>
+  </si>
+  <si>
+    <t>700g</t>
+  </si>
+  <si>
+    <t>340g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sugar </t>
+  </si>
+  <si>
+    <t>Beans</t>
   </si>
 </sst>
 </file>
@@ -512,6 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1097,8 +1527,1256 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet10"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet11"/>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet12"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet13"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet19"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet20"/>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="20.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8" t="s">
+        <v>159</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B12" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>164</v>
+      </c>
+      <c r="B13" t="s">
+        <v>155</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>164</v>
+      </c>
+      <c r="B14" t="s">
+        <v>165</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>166</v>
+      </c>
+      <c r="B15" t="s">
+        <v>166</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>167</v>
+      </c>
+      <c r="B16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>168</v>
+      </c>
+      <c r="B17" t="s">
+        <v>168</v>
+      </c>
+      <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>169</v>
+      </c>
+      <c r="B18" t="s">
+        <v>169</v>
+      </c>
+      <c r="C18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>170</v>
+      </c>
+      <c r="B19" t="s">
+        <v>170</v>
+      </c>
+      <c r="C19" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>171</v>
+      </c>
+      <c r="B20" t="s">
+        <v>174</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>172</v>
+      </c>
+      <c r="B21" t="s">
+        <v>172</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet21"/>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="29.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1264,8 +2942,338 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" t="s">
+        <v>184</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1419,6 +3427,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1499,6 +3508,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1551,8 +3561,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <sheetPr codeName="Sheet6"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1570,15 +3584,502 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" t="s">
+        <v>51</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" t="s">
+        <v>51</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" t="s">
+        <v>51</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37">
         <v>0</v>
       </c>
     </row>
@@ -1589,8 +4090,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <sheetPr codeName="Sheet7"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1608,15 +4113,695 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" t="s">
+        <v>51</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s">
+        <v>51</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>86</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B35" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" t="s">
+        <v>49</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" t="s">
+        <v>85</v>
+      </c>
+      <c r="C39" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>87</v>
+      </c>
+      <c r="B40" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" t="s">
+        <v>49</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" t="s">
+        <v>49</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>87</v>
+      </c>
+      <c r="B42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" t="s">
+        <v>49</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" t="s">
+        <v>49</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" t="s">
+        <v>49</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" t="s">
+        <v>49</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>87</v>
+      </c>
+      <c r="B46" t="s">
+        <v>20</v>
+      </c>
+      <c r="C46" t="s">
+        <v>49</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>87</v>
+      </c>
+      <c r="B47" t="s">
+        <v>30</v>
+      </c>
+      <c r="C47" t="s">
+        <v>49</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>87</v>
+      </c>
+      <c r="B48" t="s">
+        <v>31</v>
+      </c>
+      <c r="C48" t="s">
+        <v>49</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" t="s">
+        <v>89</v>
+      </c>
+      <c r="C49" t="s">
+        <v>49</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>88</v>
+      </c>
+      <c r="B50" t="s">
+        <v>18</v>
+      </c>
+      <c r="C50" t="s">
+        <v>49</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>90</v>
+      </c>
+      <c r="C51" t="s">
+        <v>49</v>
+      </c>
+      <c r="D51">
         <v>0</v>
       </c>
     </row>
@@ -1627,10 +4812,12 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D10"/>
+  <sheetPr codeName="Sheet8"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.90625" customWidth="1"/>
+    <col min="1" max="1" width="37.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -1648,58 +4835,449 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="A2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" t="s">
+        <v>107</v>
+      </c>
+      <c r="C16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>108</v>
+      </c>
+      <c r="B17" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" t="s">
+        <v>113</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet9"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
+      <c r="A5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
+      <c r="A6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
+      <c r="A7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Receipt-X v1.1.1 - Update Product Master with latest client products
</commit_message>
<xml_diff>
--- a/RECEIPT-X_PRODUCT_MASTER.xlsx
+++ b/RECEIPT-X_PRODUCT_MASTER.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8180" firstSheet="15" activeTab="22"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8180" firstSheet="35" activeTab="40"/>
   </bookViews>
   <sheets>
     <sheet name="PWANI OIL PRODUCTS" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,24 @@
     <sheet name="ZEN MAHITAJI" sheetId="28" r:id="rId21"/>
     <sheet name="SUGAR" sheetId="29" r:id="rId22"/>
     <sheet name="BEANS" sheetId="30" r:id="rId23"/>
+    <sheet name="HASBAH" sheetId="31" r:id="rId24"/>
+    <sheet name="MZAMSA" sheetId="32" r:id="rId25"/>
+    <sheet name="BHUMI" sheetId="34" r:id="rId26"/>
+    <sheet name="HIGHCHEM MARKETING" sheetId="35" r:id="rId27"/>
+    <sheet name="HIGHLANDS" sheetId="33" r:id="rId28"/>
+    <sheet name="RAISONS" sheetId="36" r:id="rId29"/>
+    <sheet name="FINSBURY" sheetId="37" r:id="rId30"/>
+    <sheet name="EXCEL CHEMICALS" sheetId="38" r:id="rId31"/>
+    <sheet name="ARAMAKARE" sheetId="51" r:id="rId32"/>
+    <sheet name="TOWFIQ" sheetId="52" r:id="rId33"/>
+    <sheet name="SRK" sheetId="54" r:id="rId34"/>
+    <sheet name="COASTAL BOTTLERS" sheetId="50" r:id="rId35"/>
+    <sheet name="RAA" sheetId="55" r:id="rId36"/>
+    <sheet name="EWCA" sheetId="56" r:id="rId37"/>
+    <sheet name="SAFWAH RESET" sheetId="57" r:id="rId38"/>
+    <sheet name="NAUSHAD TRADING" sheetId="59" r:id="rId39"/>
+    <sheet name="DP WORLD" sheetId="58" r:id="rId40"/>
+    <sheet name="LATIFA" sheetId="60" r:id="rId41"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -46,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="374">
   <si>
     <t>Brand</t>
   </si>
@@ -610,6 +628,564 @@
   </si>
   <si>
     <t>Beans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drinking chocolate sachet </t>
+  </si>
+  <si>
+    <t>Cocoa Jar</t>
+  </si>
+  <si>
+    <t>80gm</t>
+  </si>
+  <si>
+    <t>20gm 1x10doz</t>
+  </si>
+  <si>
+    <t>Drinking chocolate Jar</t>
+  </si>
+  <si>
+    <t>100gm 1x24</t>
+  </si>
+  <si>
+    <t>200gm 1x24</t>
+  </si>
+  <si>
+    <t>Nestle Nan</t>
+  </si>
+  <si>
+    <t>400gm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nescafe Classic </t>
+  </si>
+  <si>
+    <t>84x1.5gm</t>
+  </si>
+  <si>
+    <t>Always Ultra Slim</t>
+  </si>
+  <si>
+    <t>12x8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ariel Floral Fresh Clean </t>
+  </si>
+  <si>
+    <t>4x3.5kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ariel Lavender Fresh Clean </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ariel Spring Fresh Clean </t>
+  </si>
+  <si>
+    <t>Whitewash White</t>
+  </si>
+  <si>
+    <t>175gx48</t>
+  </si>
+  <si>
+    <t>Whitewash Cream</t>
+  </si>
+  <si>
+    <t>Whitewash Pink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaluma Strong Tab  </t>
+  </si>
+  <si>
+    <t>1x48g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaluma Balm </t>
+  </si>
+  <si>
+    <t>4g 1x24x24pkt</t>
+  </si>
+  <si>
+    <t>Club Soda  Orange</t>
+  </si>
+  <si>
+    <t>350mlx12</t>
+  </si>
+  <si>
+    <t>Club Soda  Lemon</t>
+  </si>
+  <si>
+    <t>Club Soda  Pineapple</t>
+  </si>
+  <si>
+    <t>Club Soda  Cola</t>
+  </si>
+  <si>
+    <t>Club Soda  Black Vurrant</t>
+  </si>
+  <si>
+    <t>Club Soda  Tangawizi</t>
+  </si>
+  <si>
+    <t>Tidex Serviette Yellow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clown Pan Masala  </t>
+  </si>
+  <si>
+    <t>20x80pcs</t>
+  </si>
+  <si>
+    <t>Virani Curry Powder</t>
+  </si>
+  <si>
+    <t>12x24x10g</t>
+  </si>
+  <si>
+    <t>Weetabix Single</t>
+  </si>
+  <si>
+    <t>37gx24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sevin DUDU dUST  </t>
+  </si>
+  <si>
+    <t>24X200gm</t>
+  </si>
+  <si>
+    <t>Riza Basmati Long Grain Rice</t>
+  </si>
+  <si>
+    <t>1x20kg</t>
+  </si>
+  <si>
+    <t>KSL Tropical Mints</t>
+  </si>
+  <si>
+    <t>12x500gms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anfa Energy Chocolate </t>
+  </si>
+  <si>
+    <t>120x33</t>
+  </si>
+  <si>
+    <t>Anfa Energy Milk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunveat Vanilla Cream </t>
+  </si>
+  <si>
+    <t>60pkts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunveat Pineapple  Cream </t>
+  </si>
+  <si>
+    <t>Sunveat Orange Cream</t>
+  </si>
+  <si>
+    <t>Golden Ginger Nut Carton</t>
+  </si>
+  <si>
+    <t>60x3pcs</t>
+  </si>
+  <si>
+    <t>Biz Razor Pouch</t>
+  </si>
+  <si>
+    <t>1ctn=8 Outers</t>
+  </si>
+  <si>
+    <t>Sunveat Strawberry Cream</t>
+  </si>
+  <si>
+    <t>Sunveat Chocolate Cream</t>
+  </si>
+  <si>
+    <t>Sunveat Mango Cream</t>
+  </si>
+  <si>
+    <t>Nice</t>
+  </si>
+  <si>
+    <t>60gx36pkts</t>
+  </si>
+  <si>
+    <t>Kreams Gold Strawberry</t>
+  </si>
+  <si>
+    <t>11gmsx60pkts</t>
+  </si>
+  <si>
+    <t>Kreams Gold Chocolate</t>
+  </si>
+  <si>
+    <t>Kreams Gold Vanilla</t>
+  </si>
+  <si>
+    <t>Ginger snap</t>
+  </si>
+  <si>
+    <t>12gmsx60pkts</t>
+  </si>
+  <si>
+    <t>Milk power Choco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nice </t>
+  </si>
+  <si>
+    <t>10gmx72pkts</t>
+  </si>
+  <si>
+    <t>Milk Power</t>
+  </si>
+  <si>
+    <t>Cowboy</t>
+  </si>
+  <si>
+    <t>Msafi Lavender Fresh</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 200g Sachet</t>
+  </si>
+  <si>
+    <t>Msafi Purple Fresh</t>
+  </si>
+  <si>
+    <t>Pep Rose Concentrate</t>
+  </si>
+  <si>
+    <t>Champ RTD Orange</t>
+  </si>
+  <si>
+    <t>500g24x150ml</t>
+  </si>
+  <si>
+    <t>Gofruit Assorted Pack</t>
+  </si>
+  <si>
+    <t>12x250ml</t>
+  </si>
+  <si>
+    <t>Excel Raha Drinking Chocolate</t>
+  </si>
+  <si>
+    <t>144x8gms</t>
+  </si>
+  <si>
+    <t>96x16gm</t>
+  </si>
+  <si>
+    <t>Eveready H Duty AAA Red</t>
+  </si>
+  <si>
+    <t>10x2</t>
+  </si>
+  <si>
+    <t>Red Bull Energy Drink</t>
+  </si>
+  <si>
+    <t>250ml</t>
+  </si>
+  <si>
+    <t>Zain</t>
+  </si>
+  <si>
+    <t>20lts</t>
+  </si>
+  <si>
+    <t>10lts</t>
+  </si>
+  <si>
+    <t>Predator Gold Strike</t>
+  </si>
+  <si>
+    <t>400ml</t>
+  </si>
+  <si>
+    <t>Be Olive Oil Cleansing And Moisturizing Shampoo(2 in 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Be Olive Oil Cleansing And MoisturizingEgg  Shampoo(2 in 1) </t>
+  </si>
+  <si>
+    <t>Be Olive Oil Cleansing And Moisturizing  Shampoo (2 in 1)</t>
+  </si>
+  <si>
+    <t>Be Olive Oil Cleansing And Moisturizing Egg Shampoo(2 in 1)</t>
+  </si>
+  <si>
+    <t>Jik Bleach Regular</t>
+  </si>
+  <si>
+    <t>70ml x144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strepsils Regular </t>
+  </si>
+  <si>
+    <t>50x2(24unit)</t>
+  </si>
+  <si>
+    <t>Strepsils Honey &amp; Lemon</t>
+  </si>
+  <si>
+    <t>Mortein D/P .Guard AIK Lemon</t>
+  </si>
+  <si>
+    <t>12x100ml</t>
+  </si>
+  <si>
+    <t>Dettol Soap Cool</t>
+  </si>
+  <si>
+    <t>72x60g</t>
+  </si>
+  <si>
+    <t>Dettol Soap Herbal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dettol Soap ORG </t>
+  </si>
+  <si>
+    <t xml:space="preserve">85G </t>
+  </si>
+  <si>
+    <t>60g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harpic Power Plus </t>
+  </si>
+  <si>
+    <t>30pcs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Princess Pink Chicken 9g Togs </t>
+  </si>
+  <si>
+    <t>Princess Pink Tomato 9g with Toys</t>
+  </si>
+  <si>
+    <t>Princess BBQ flavor 9g with Toys</t>
+  </si>
+  <si>
+    <t>Fun-Time Tomato Flavour 9g Toys</t>
+  </si>
+  <si>
+    <t>Fun-Time Chicken Flavour 9g Toys</t>
+  </si>
+  <si>
+    <t>Kids Fun Balloon Joy Chicken Flavour 9g Toys</t>
+  </si>
+  <si>
+    <t>Kids Fun Balloon Joy BBQ Flavour 9g Toys</t>
+  </si>
+  <si>
+    <t>Kids Fun Balloon Joy Tomato Flavour 9g Toys</t>
+  </si>
+  <si>
+    <t>Kids Fun Back To School BBQ flavor With Gifts 9g</t>
+  </si>
+  <si>
+    <t>Kids Fun Back To School CHK flavor With Gifts 9g</t>
+  </si>
+  <si>
+    <t>Kids Fun Back To School TOM  flavor With Gifts 9g</t>
+  </si>
+  <si>
+    <t>Yummy Yellow Chicken 9g Toys</t>
+  </si>
+  <si>
+    <t>Kids Fun Car &amp; Bike Tomato Flavour 9g</t>
+  </si>
+  <si>
+    <t>Kids Fun Car &amp; Bike ChickenFlavour 9g</t>
+  </si>
+  <si>
+    <t>Kids Fun Car &amp; Bike BBQ Flavour 9g</t>
+  </si>
+  <si>
+    <t>50x2</t>
+  </si>
+  <si>
+    <t>Menthoking 18pkts</t>
+  </si>
+  <si>
+    <t>Menthoking Plus</t>
+  </si>
+  <si>
+    <t>9ml</t>
+  </si>
+  <si>
+    <t>Crunchy Toys Tomato</t>
+  </si>
+  <si>
+    <t>Crunchy Toys Chicken</t>
+  </si>
+  <si>
+    <t>Bale</t>
+  </si>
+  <si>
+    <t>Glint Natural Dream</t>
+  </si>
+  <si>
+    <t>Roll on</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glint Tender </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glint Magic </t>
+  </si>
+  <si>
+    <t>Glint Power</t>
+  </si>
+  <si>
+    <t>Glint Thermic</t>
+  </si>
+  <si>
+    <t>Glint Protec</t>
+  </si>
+  <si>
+    <t>Glint Cool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eno Tabs  </t>
+  </si>
+  <si>
+    <t>48s</t>
+  </si>
+  <si>
+    <t>Eno Cal Antacid Tabs</t>
+  </si>
+  <si>
+    <t>Panadol Extra Optizorb</t>
+  </si>
+  <si>
+    <t>100s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panadol Advance </t>
+  </si>
+  <si>
+    <t>Eno Lemon</t>
+  </si>
+  <si>
+    <t>24s</t>
+  </si>
+  <si>
+    <t>GBK  Star Cream Choco</t>
+  </si>
+  <si>
+    <t>60x2pcs</t>
+  </si>
+  <si>
+    <t>Huggies Baby Essentials</t>
+  </si>
+  <si>
+    <t>48x6</t>
+  </si>
+  <si>
+    <t>42X6</t>
+  </si>
+  <si>
+    <t>40X6</t>
+  </si>
+  <si>
+    <t>36X6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rice </t>
+  </si>
+  <si>
+    <t>25kgs</t>
+  </si>
+  <si>
+    <t>Al-Hakim Rice</t>
+  </si>
+  <si>
+    <t>20kg</t>
+  </si>
+  <si>
+    <t>Straw Soda</t>
+  </si>
+  <si>
+    <t>Adix Pen Blue</t>
+  </si>
+  <si>
+    <t>Adix Pen Black</t>
+  </si>
+  <si>
+    <t>Adix Pen Red</t>
+  </si>
+  <si>
+    <t>Vastline powder</t>
+  </si>
+  <si>
+    <t>Gazetti</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>Macorononi Big Elbow</t>
+  </si>
+  <si>
+    <t>Ctn</t>
+  </si>
+  <si>
+    <t>Pasta Savana</t>
+  </si>
+  <si>
+    <t>Sunrice</t>
+  </si>
+  <si>
+    <t>Diclofenac</t>
+  </si>
+  <si>
+    <t>Kleenshave Wembe</t>
+  </si>
+  <si>
+    <t>Samaki Hilwa Kubwa</t>
+  </si>
+  <si>
+    <t>Samaki Hilwa Ndogo</t>
+  </si>
+  <si>
+    <t>Gas Lighter</t>
+  </si>
+  <si>
+    <t>Chest Cof Tablets</t>
+  </si>
+  <si>
+    <t>Ear Buds</t>
+  </si>
+  <si>
+    <t>Baba Rice</t>
+  </si>
+  <si>
+    <t>Al Taam Rice</t>
+  </si>
+  <si>
+    <t>Yeast Bakerdream</t>
+  </si>
+  <si>
+    <t>11g</t>
+  </si>
+  <si>
+    <t>Candles</t>
+  </si>
+  <si>
+    <t>ctn</t>
+  </si>
+  <si>
+    <t>pcs</t>
+  </si>
+  <si>
+    <t>Pcs</t>
   </si>
 </sst>
 </file>
@@ -942,10 +1518,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.1796875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -1519,6 +2096,48 @@
         <v>49</v>
       </c>
       <c r="D41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D44">
         <v>0</v>
       </c>
     </row>
@@ -1554,6 +2173,9 @@
       <c r="A2" t="s">
         <v>119</v>
       </c>
+      <c r="B2" t="s">
+        <v>373</v>
+      </c>
       <c r="C2" t="s">
         <v>51</v>
       </c>
@@ -1565,6 +2187,9 @@
       <c r="A3" t="s">
         <v>120</v>
       </c>
+      <c r="B3" t="s">
+        <v>373</v>
+      </c>
       <c r="C3" t="s">
         <v>49</v>
       </c>
@@ -1576,6 +2201,9 @@
       <c r="A4" t="s">
         <v>121</v>
       </c>
+      <c r="B4" t="s">
+        <v>373</v>
+      </c>
       <c r="C4" t="s">
         <v>49</v>
       </c>
@@ -1587,6 +2215,9 @@
       <c r="A5" t="s">
         <v>122</v>
       </c>
+      <c r="B5" t="s">
+        <v>373</v>
+      </c>
       <c r="C5" t="s">
         <v>49</v>
       </c>
@@ -1598,6 +2229,9 @@
       <c r="A6" t="s">
         <v>123</v>
       </c>
+      <c r="B6" t="s">
+        <v>373</v>
+      </c>
       <c r="C6" t="s">
         <v>49</v>
       </c>
@@ -1608,6 +2242,9 @@
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>124</v>
+      </c>
+      <c r="B7" t="s">
+        <v>373</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
@@ -2777,7 +3414,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" customWidth="1"/>
@@ -2934,6 +3571,48 @@
         <v>49</v>
       </c>
       <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14">
         <v>0</v>
       </c>
     </row>
@@ -3271,6 +3950,692 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B10" t="s">
+        <v>202</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>204</v>
+      </c>
+      <c r="B11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>271</v>
+      </c>
+      <c r="B12" t="s">
+        <v>272</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>273</v>
+      </c>
+      <c r="B13" t="s">
+        <v>274</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B3" t="s">
+        <v>212</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B4" t="s">
+        <v>372</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>217</v>
+      </c>
+      <c r="B5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>218</v>
+      </c>
+      <c r="B6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>219</v>
+      </c>
+      <c r="B7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B4" t="s">
+        <v>234</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>235</v>
+      </c>
+      <c r="B5" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>239</v>
+      </c>
+      <c r="B8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B9" t="s">
+        <v>241</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B10" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>244</v>
+      </c>
+      <c r="B11" t="s">
+        <v>237</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>245</v>
+      </c>
+      <c r="B12" t="s">
+        <v>237</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>246</v>
+      </c>
+      <c r="B13" t="s">
+        <v>237</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet3"/>
@@ -3419,6 +4784,1023 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C11" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>263</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>266</v>
+      </c>
+      <c r="B3" t="s">
+        <v>267</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>268</v>
+      </c>
+      <c r="B5" t="s">
+        <v>270</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="51.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>282</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>280</v>
+      </c>
+      <c r="B5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>288</v>
+      </c>
+      <c r="B4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>291</v>
+      </c>
+      <c r="B6" t="s">
+        <v>292</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>293</v>
+      </c>
+      <c r="B7" t="s">
+        <v>292</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>294</v>
+      </c>
+      <c r="B8" t="s">
+        <v>295</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>293</v>
+      </c>
+      <c r="B9" t="s">
+        <v>295</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>294</v>
+      </c>
+      <c r="B10" t="s">
+        <v>296</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>284</v>
+      </c>
+      <c r="B11" t="s">
+        <v>274</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>297</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>297</v>
+      </c>
+      <c r="B13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="41.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>300</v>
+      </c>
+      <c r="B3" t="s">
+        <v>298</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>301</v>
+      </c>
+      <c r="B4" t="s">
+        <v>298</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>302</v>
+      </c>
+      <c r="B5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>303</v>
+      </c>
+      <c r="B6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>304</v>
+      </c>
+      <c r="B7" t="s">
+        <v>298</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>306</v>
+      </c>
+      <c r="B9" t="s">
+        <v>298</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>307</v>
+      </c>
+      <c r="B10" t="s">
+        <v>298</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>308</v>
+      </c>
+      <c r="B11" t="s">
+        <v>298</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>309</v>
+      </c>
+      <c r="B12" t="s">
+        <v>298</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>310</v>
+      </c>
+      <c r="B13" t="s">
+        <v>298</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>311</v>
+      </c>
+      <c r="B14" t="s">
+        <v>298</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>312</v>
+      </c>
+      <c r="B15" t="s">
+        <v>298</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>313</v>
+      </c>
+      <c r="B16" t="s">
+        <v>298</v>
+      </c>
+      <c r="C16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>315</v>
+      </c>
+      <c r="B2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>319</v>
+      </c>
+      <c r="B3" t="s">
+        <v>320</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>321</v>
+      </c>
+      <c r="B3" t="s">
+        <v>322</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>325</v>
+      </c>
+      <c r="B5" t="s">
+        <v>322</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>326</v>
+      </c>
+      <c r="B6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B7" t="s">
+        <v>322</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>328</v>
+      </c>
+      <c r="B8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B2" t="s">
+        <v>345</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3506,11 +5888,588 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>331</v>
+      </c>
+      <c r="B3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>332</v>
+      </c>
+      <c r="B4" t="s">
+        <v>333</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>334</v>
+      </c>
+      <c r="B5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>337</v>
+      </c>
+      <c r="B7" t="s">
+        <v>338</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>337</v>
+      </c>
+      <c r="B8" t="s">
+        <v>338</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>337</v>
+      </c>
+      <c r="B9" t="s">
+        <v>338</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>339</v>
+      </c>
+      <c r="B10" t="s">
+        <v>340</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>339</v>
+      </c>
+      <c r="B11" t="s">
+        <v>341</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>339</v>
+      </c>
+      <c r="B12" t="s">
+        <v>342</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>339</v>
+      </c>
+      <c r="B13" t="s">
+        <v>343</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>348</v>
+      </c>
+      <c r="B3" t="s">
+        <v>371</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B5" t="s">
+        <v>371</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>351</v>
+      </c>
+      <c r="B6" t="s">
+        <v>371</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>352</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>353</v>
+      </c>
+      <c r="B8" t="s">
+        <v>354</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>355</v>
+      </c>
+      <c r="B9" t="s">
+        <v>356</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>357</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>358</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>358</v>
+      </c>
+      <c r="B12" t="s">
+        <v>347</v>
+      </c>
+      <c r="C12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>358</v>
+      </c>
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>358</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>358</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>359</v>
+      </c>
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>360</v>
+      </c>
+      <c r="B17" t="s">
+        <v>372</v>
+      </c>
+      <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>361</v>
+      </c>
+      <c r="B18" t="s">
+        <v>371</v>
+      </c>
+      <c r="C18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>362</v>
+      </c>
+      <c r="B19" t="s">
+        <v>371</v>
+      </c>
+      <c r="C19" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>363</v>
+      </c>
+      <c r="B20" t="s">
+        <v>371</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>364</v>
+      </c>
+      <c r="B21" t="s">
+        <v>371</v>
+      </c>
+      <c r="C21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>365</v>
+      </c>
+      <c r="B22" t="s">
+        <v>372</v>
+      </c>
+      <c r="C22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>366</v>
+      </c>
+      <c r="B23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>367</v>
+      </c>
+      <c r="B24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>368</v>
+      </c>
+      <c r="B25" t="s">
+        <v>369</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>370</v>
+      </c>
+      <c r="B26" t="s">
+        <v>371</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -3551,6 +6510,118 @@
         <v>49</v>
       </c>
       <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>249</v>
+      </c>
+      <c r="B5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>251</v>
+      </c>
+      <c r="B6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>255</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>256</v>
+      </c>
+      <c r="B10" t="s">
+        <v>257</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>258</v>
+      </c>
+      <c r="B11" t="s">
+        <v>257</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
         <v>0</v>
       </c>
     </row>
@@ -4075,6 +7146,9 @@
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>65</v>
+      </c>
+      <c r="B37" t="s">
+        <v>354</v>
       </c>
       <c r="C37" t="s">
         <v>51</v>

</xml_diff>